<commit_message>
Update AI5 -PUBLIC content
</commit_message>
<xml_diff>
--- a/AI5 -PUBLIC/Videos.xlsx
+++ b/AI5 -PUBLIC/Videos.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="20">
   <si>
     <t>Lesson no</t>
   </si>
@@ -40,6 +40,43 @@
   </si>
   <si>
     <t xml:space="preserve">Lesson  3 </t>
+  </si>
+  <si>
+    <t>Lesson  4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lesson 5 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://us02web.zoom.us/rec/share/NjpfXyvBj-Z1_TIgw6WauJ9g-Kyc4xmNMgGOttmX634nsUyLJLAnlltxZa61kYOz.MQlFm1ILOf2ydMO- 
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lesson 7 </t>
+  </si>
+  <si>
+    <t>Lesson 8</t>
+  </si>
+  <si>
+    <t>8K0s@LhU</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lesson 9 </t>
+  </si>
+  <si>
+    <t>Lesson  10</t>
+  </si>
+  <si>
+    <t>Lesson 11</t>
+  </si>
+  <si>
+    <t>cTBJ8#rV</t>
+  </si>
+  <si>
+    <t>סדנת חיפוש עבודה</t>
+  </si>
+  <si>
+    <t>J@p2!i#$</t>
   </si>
 </sst>
 </file>
@@ -71,14 +108,14 @@
       <name val="Helvetica Neue"/>
     </font>
     <font>
-      <sz val="10.0"/>
-      <color rgb="FF1155CC"/>
+      <color theme="1"/>
       <name val="Arial"/>
+      <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10.0"/>
-      <color rgb="FF44BBFF"/>
-      <name val="Helvetica Neue"/>
+      <u/>
+      <sz val="11.0"/>
+      <color rgb="FF0000FF"/>
     </font>
   </fonts>
   <fills count="4">
@@ -113,7 +150,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="8">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -122,27 +159,20 @@
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="1" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center"/>
+      <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -385,93 +415,167 @@
       <c r="D5" s="3">
         <v>1.0</v>
       </c>
-      <c r="E5" s="4">
+      <c r="E5" s="3">
         <v>23.11</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="F5" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="G5" s="3" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="6" ht="15.75" customHeight="1">
-      <c r="D6" s="4">
+      <c r="D6" s="3">
         <v>2.0</v>
       </c>
-      <c r="E6" s="4">
+      <c r="E6" s="3">
         <v>30.11</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="F6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="G6" s="3" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="7" ht="15.75" customHeight="1">
-      <c r="D7" s="4">
+      <c r="D7" s="3">
         <v>3.0</v>
       </c>
-      <c r="E7" s="4">
+      <c r="E7" s="3">
         <v>7.12</v>
       </c>
-      <c r="F7" s="5" t="s">
+      <c r="F7" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="G7" s="4" t="s">
+      <c r="G7" s="3" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="8" ht="15.75" customHeight="1">
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="8"/>
-      <c r="G8" s="7"/>
+      <c r="D8" s="3">
+        <v>4.0</v>
+      </c>
+      <c r="E8" s="3">
+        <v>21.12</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="9" ht="15.75" customHeight="1">
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="9"/>
-      <c r="G9" s="7"/>
+      <c r="D9" s="3">
+        <v>5.0</v>
+      </c>
+      <c r="E9" s="3">
+        <v>28.12</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="10" ht="15.75" customHeight="1">
-      <c r="D10" s="7"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="10"/>
-      <c r="G10" s="7"/>
+      <c r="D10" s="3">
+        <v>6.0</v>
+      </c>
+      <c r="E10" s="3">
+        <v>4.1</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="11" ht="15.75" customHeight="1">
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
-      <c r="G11" s="7"/>
+      <c r="D11" s="3">
+        <v>7.0</v>
+      </c>
+      <c r="E11" s="3">
+        <v>11.1</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="12" ht="15.75" customHeight="1">
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="7"/>
+      <c r="D12" s="3">
+        <v>8.0</v>
+      </c>
+      <c r="E12" s="3">
+        <v>18.1</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="13" ht="15.75" customHeight="1">
-      <c r="D13" s="7"/>
-      <c r="E13" s="7"/>
-      <c r="F13" s="7"/>
-      <c r="G13" s="7"/>
+      <c r="D13" s="3">
+        <v>9.0</v>
+      </c>
+      <c r="E13" s="3">
+        <v>25.1</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="14" ht="15.75" customHeight="1">
-      <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7"/>
-      <c r="G14" s="7"/>
+      <c r="D14" s="3">
+        <v>10.0</v>
+      </c>
+      <c r="E14" s="3">
+        <v>1.2</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="15" ht="15.75" customHeight="1">
-      <c r="D15" s="7"/>
-      <c r="E15" s="7"/>
-      <c r="F15" s="7"/>
-      <c r="G15" s="7"/>
+      <c r="D15" s="3">
+        <v>11.0</v>
+      </c>
+      <c r="E15" s="3">
+        <v>8.2</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
-    <row r="16" ht="15.75" customHeight="1"/>
+    <row r="16" ht="15.75" customHeight="1">
+      <c r="E16" s="6">
+        <v>24.2</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="G16" s="6" t="s">
+        <v>19</v>
+      </c>
+    </row>
     <row r="17" ht="15.75" customHeight="1"/>
     <row r="18" ht="15.75" customHeight="1"/>
     <row r="19" ht="15.75" customHeight="1"/>
@@ -1461,10 +1565,19 @@
     <hyperlink r:id="rId1" ref="F5"/>
     <hyperlink r:id="rId2" ref="F6"/>
     <hyperlink r:id="rId3" ref="F7"/>
+    <hyperlink r:id="rId4" ref="F8"/>
+    <hyperlink r:id="rId5" ref="F9"/>
+    <hyperlink r:id="rId6" ref="F10"/>
+    <hyperlink r:id="rId7" ref="F11"/>
+    <hyperlink r:id="rId8" ref="F12"/>
+    <hyperlink r:id="rId9" ref="F13"/>
+    <hyperlink r:id="rId10" ref="F14"/>
+    <hyperlink r:id="rId11" ref="F15"/>
+    <hyperlink r:id="rId12" ref="F16"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId4"/>
+  <drawing r:id="rId13"/>
 </worksheet>
 </file>
</xml_diff>